<commit_message>
claudecode fiksa find_wave_range, noe mer må gjøres, ligger som TODO
</commit_message>
<xml_diff>
--- a/waveprocessed/PROCESSED-20251112-tett6roof-lowM-579komma8/meta.xlsx
+++ b/waveprocessed/PROCESSED-20251112-tett6roof-lowM-579komma8/meta.xlsx
@@ -1219,47 +1219,47 @@
         <v>271.77536</v>
       </c>
       <c r="P3" t="n">
-        <v>4700</v>
+        <v>4765</v>
       </c>
       <c r="Q3" t="n">
-        <v>9315.384615384615</v>
+        <v>9385</v>
       </c>
       <c r="R3" t="n">
         <v>8.164999999999992</v>
       </c>
       <c r="S3" t="n">
-        <v>7.672435294646441</v>
+        <v>7.668165556097218</v>
       </c>
       <c r="T3" t="n">
-        <v>7.66935138540088</v>
+        <v>7.671622195108402</v>
       </c>
       <c r="U3" t="n">
-        <v>10.86023957826251</v>
+        <v>10.86203518503066</v>
       </c>
       <c r="V3" t="n">
-        <v>0.5488201436566842</v>
+        <v>0.5444774348407886</v>
       </c>
       <c r="W3" t="n">
-        <v>10.87409799695325</v>
+        <v>10.87567303838686</v>
       </c>
       <c r="X3" t="n">
-        <v>0.7693333333333332</v>
+        <v>0.7701666666666668</v>
       </c>
       <c r="Y3" t="n">
-        <v>6.80664920385966</v>
+        <v>6.792013952800097</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.9230952145464986</v>
+        <v>0.9250842755688481</v>
       </c>
       <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="n">
-        <v>0.05557629074951407</v>
+        <v>0.05545679392461274</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.9992556045629514</v>
+        <v>0.9992428639850438</v>
       </c>
       <c r="AD3" t="n">
-        <v>1.199863797070839</v>
+        <v>1.201148161309909</v>
       </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
@@ -1270,47 +1270,47 @@
         <v>272.17708</v>
       </c>
       <c r="AI3" t="n">
-        <v>4800</v>
+        <v>4890</v>
       </c>
       <c r="AJ3" t="n">
-        <v>9415.384615384615</v>
+        <v>9511</v>
       </c>
       <c r="AK3" t="n">
-        <v>8.164625000000019</v>
+        <v>8.115799999999986</v>
       </c>
       <c r="AL3" t="n">
-        <v>7.549961957250483</v>
+        <v>7.52489746119665</v>
       </c>
       <c r="AM3" t="n">
-        <v>7.556112302260837</v>
+        <v>7.555524875248878</v>
       </c>
       <c r="AN3" t="n">
-        <v>10.70199360102871</v>
+        <v>10.69995048830427</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.5741199846569051</v>
+        <v>0.5674615774962207</v>
       </c>
       <c r="AP3" t="n">
-        <v>10.71738218004947</v>
+        <v>10.71498731189623</v>
       </c>
       <c r="AQ3" t="n">
-        <v>0.7693333333333332</v>
+        <v>0.7703333333333333</v>
       </c>
       <c r="AR3" t="n">
-        <v>6.80664920385966</v>
+        <v>6.789092731771488</v>
       </c>
       <c r="AS3" t="n">
-        <v>0.9230952145464986</v>
+        <v>0.9254823222218833</v>
       </c>
       <c r="AT3" t="inlineStr"/>
       <c r="AU3" t="n">
-        <v>0.05557373825606281</v>
+        <v>0.05509891879251094</v>
       </c>
       <c r="AV3" t="n">
-        <v>0.9992556045629514</v>
+        <v>0.9992402949658459</v>
       </c>
       <c r="AW3" t="n">
-        <v>1.199863797070839</v>
+        <v>1.20140500504788</v>
       </c>
       <c r="AX3" t="inlineStr"/>
       <c r="AY3" t="inlineStr"/>
@@ -1321,47 +1321,47 @@
         <v>272.19024</v>
       </c>
       <c r="BB3" t="n">
-        <v>6500</v>
+        <v>6476</v>
       </c>
       <c r="BC3" t="n">
-        <v>11115.38461538462</v>
+        <v>11096</v>
       </c>
       <c r="BD3" t="n">
         <v>8.20999999999998</v>
       </c>
       <c r="BE3" t="n">
-        <v>7.463072723853617</v>
+        <v>7.448246623149639</v>
       </c>
       <c r="BF3" t="n">
-        <v>7.457623089896896</v>
+        <v>7.458229989921048</v>
       </c>
       <c r="BG3" t="n">
-        <v>10.56833973741926</v>
+        <v>10.56801689527296</v>
       </c>
       <c r="BH3" t="n">
-        <v>0.7673875096728714</v>
+        <v>0.7678072332717274</v>
       </c>
       <c r="BI3" t="n">
-        <v>10.59616385280621</v>
+        <v>10.59587226453014</v>
       </c>
       <c r="BJ3" t="n">
-        <v>0.7693333333333332</v>
+        <v>0.7701666666666668</v>
       </c>
       <c r="BK3" t="n">
-        <v>6.80664920385966</v>
+        <v>6.792013952800097</v>
       </c>
       <c r="BL3" t="n">
-        <v>0.9230952145464986</v>
+        <v>0.9250842755688481</v>
       </c>
       <c r="BM3" t="inlineStr"/>
       <c r="BN3" t="n">
-        <v>0.05588258996368767</v>
+        <v>0.05576243455248866</v>
       </c>
       <c r="BO3" t="n">
-        <v>0.9992556045629514</v>
+        <v>0.9992428639850438</v>
       </c>
       <c r="BP3" t="n">
-        <v>1.199863797070839</v>
+        <v>1.201148161309909</v>
       </c>
       <c r="BQ3" t="inlineStr"/>
       <c r="BR3" t="inlineStr"/>
@@ -1372,47 +1372,47 @@
         <v>273.01376</v>
       </c>
       <c r="BU3" t="n">
-        <v>6500</v>
+        <v>6479</v>
       </c>
       <c r="BV3" t="n">
-        <v>11115.38461538462</v>
+        <v>11099</v>
       </c>
       <c r="BW3" t="n">
         <v>8.204999999999984</v>
       </c>
       <c r="BX3" t="n">
-        <v>7.559439166637769</v>
+        <v>7.545937008563378</v>
       </c>
       <c r="BY3" t="n">
-        <v>7.526144785668698</v>
+        <v>7.525865963653561</v>
       </c>
       <c r="BZ3" t="n">
-        <v>10.66354571414305</v>
+        <v>10.66211227128651</v>
       </c>
       <c r="CA3" t="n">
-        <v>0.6961717896805124</v>
+        <v>0.69723359473877</v>
       </c>
       <c r="CB3" t="n">
-        <v>10.68624641108212</v>
+        <v>10.68488524838478</v>
       </c>
       <c r="CC3" t="n">
-        <v>0.7693333333333332</v>
+        <v>0.7701666666666668</v>
       </c>
       <c r="CD3" t="n">
-        <v>6.80664920385966</v>
+        <v>6.792013952800097</v>
       </c>
       <c r="CE3" t="n">
-        <v>0.9230952145464986</v>
+        <v>0.9250842755688481</v>
       </c>
       <c r="CF3" t="inlineStr"/>
       <c r="CG3" t="n">
-        <v>0.0558485567176684</v>
+        <v>0.05572847448272469</v>
       </c>
       <c r="CH3" t="n">
-        <v>0.9992556045629514</v>
+        <v>0.9992428639850438</v>
       </c>
       <c r="CI3" t="n">
-        <v>1.199863797070839</v>
+        <v>1.201148161309909</v>
       </c>
       <c r="CJ3" t="inlineStr"/>
       <c r="CK3" t="inlineStr"/>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="CO3" t="inlineStr"/>
       <c r="CP3" t="n">
-        <v>0.05558847234284223</v>
+        <v>0.05525604958464561</v>
       </c>
       <c r="CQ3" t="n">
         <v>3.948903220766223</v>
@@ -1444,25 +1444,25 @@
       </c>
       <c r="CX3" t="inlineStr"/>
       <c r="CY3" t="n">
-        <v>0.9840372277259327</v>
+        <v>0.9813165099458956</v>
       </c>
       <c r="CZ3" t="n">
-        <v>0.9884914342762452</v>
+        <v>0.9898137033172514</v>
       </c>
       <c r="DA3" t="n">
-        <v>1.012912435179165</v>
+        <v>1.013115890270082</v>
       </c>
       <c r="DB3" t="n">
-        <v>1.299826689774697</v>
+        <v>1.298420255355983</v>
       </c>
       <c r="DC3" t="n">
-        <v>1.299826689774697</v>
+        <v>1.298139333621809</v>
       </c>
       <c r="DD3" t="n">
-        <v>1.299826689774697</v>
+        <v>1.298420255355983</v>
       </c>
       <c r="DE3" t="n">
-        <v>1.299826689774697</v>
+        <v>1.298420255355983</v>
       </c>
       <c r="DF3" t="inlineStr">
         <is>

</xml_diff>